<commit_message>
vault backup: 2026-07-09 15:35:22
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件概要设计-模块功能拆分.xlsx
+++ b/公司项目/认知作战/文档/软件概要设计-模块功能拆分.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="32400" windowHeight="18375" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12420" firstSheet="2" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="模块清单总览" sheetId="1" r:id="rId1"/>
@@ -3220,7 +3220,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3242,6 +3242,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3577,7 +3583,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
@@ -3601,16 +3607,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="6">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="5">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="7">
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="7">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="8">
@@ -3619,89 +3625,89 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3719,6 +3725,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9848,7 +9857,7 @@
       <c r="A19" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>923</v>
       </c>
       <c r="C19" s="6" t="s">
@@ -9874,7 +9883,7 @@
       <c r="A20" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="7" t="s">
         <v>928</v>
       </c>
       <c r="C20" s="6" t="s">
@@ -9900,7 +9909,7 @@
       <c r="A21" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>932</v>
       </c>
       <c r="C21" s="6" t="s">
@@ -9926,7 +9935,7 @@
       <c r="A22" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="7" t="s">
         <v>936</v>
       </c>
       <c r="C22" s="6" t="s">
@@ -9952,7 +9961,7 @@
       <c r="A23" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>940</v>
       </c>
       <c r="C23" s="6" t="s">

</xml_diff>

<commit_message>
vault backup: 2026-07-09 16:36:06
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件概要设计-模块功能拆分.xlsx
+++ b/公司项目/认知作战/文档/软件概要设计-模块功能拆分.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -195,6 +195,9 @@
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="37">
@@ -415,7 +418,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -535,6 +538,20 @@
         <color theme="4"/>
       </bottom>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="49">
@@ -684,7 +701,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -705,6 +722,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7453,7 +7473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="18"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8336,7 +8356,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>F-SWM-06-01 有效性评测(线上MC作业效果统计)；F-SWM-06-02 稳定性与合规性评估(离线数据集benchmark评测)；F-SWM-06-03 迭代/淘汰决策与反馈闭环</t>
+          <t>F-SWM-06-01 有效性评测(线上MC作业效果统计)；F-SWM-06-02 评测数据集管理；F-SWM-06-03 批量跑题执行；F-SWM-06-04 答案对比与打分；F-SWM-06-05 评分汇总与报告；F-SWM-06-06 迭代/淘汰决策与反馈闭环</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -8346,7 +8366,7 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>对应 R-SWM-004。06-01 为线上效果统计(触达/互动/完成率)、06-02 为离线数据集评测(标准题集+预期答案+对比打分)，一在线一离线互补评估智能体质量；决策与反馈(06-03)内聚不拆。</t>
+          <t>对应 R-SWM-004。06-01 为线上效果统计(触达/互动/完成率)；06-02~05 为离线数据集评测流程(录入题集→跑题→打分→汇总)，按流程环节拆4个功能；一在线一离线互补评估；06-06 综合双轨结论做决策与反馈。</t>
         </is>
       </c>
     </row>
@@ -8393,84 +8413,210 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>F-SWM-06-02</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>稳定性与合规性评估</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>评测数据集管理</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>R-SWM-004</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>基于标准评测数据集（人工编辑的测试题集，含问题+预期答案+评分维度）对智能体进行离线 benchmark 评测：批量跑题收集实际回答 → 对比预期答案打分 → 按稳定性/合规性/人设一致性维度汇总得分，评估智能体在受控测试集上的表现质量。</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>评测数据集录入与管理(问题/预期答案/评分维度)；批量执行评测(跑题,调用SWM定义+IRS推理收集回答)；答案对比与打分(人工评判/规则匹配/LLM-as-judge)；评分汇总与报告(稳定性/合规性/人设一致性得分)</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>SRS R-SWM-004；离线数据集评测</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>数据来自 R-MC-008</t>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>管理智能体评测用的标准数据集：提示词工程师编辑测试用例集，每条用例含问题、预期答案、评分标准（规则匹配/关键词/LLM裁判/人工评判）、权重与所属评分维度（稳定性/合规性/人设一致性）；支持数据集创建、用例录入/批量导入/修改/删除与版本管理。</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>数据集创建与元信息(适用人设/评分维度)；用例录入(问题/预期答案/评分标准/权重/维度)；批量导入；用例增删改查；数据集版本管理</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>SRS R-SWM-004</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>数据集是离线评测的可复现基准，固定题集可对不同版本反复评测对比演进</t>
         </is>
       </c>
     </row>
     <row r="25" ht="33" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>F-SWM-06-03</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>批量跑题执行</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>R-SWM-004</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>对指定 agent_id 按数据集逐题执行评测：系统将每题问题连同智能体定义（提示词+人设+记忆）交由 IRS 本地大模型推理（不经执行网关），收集智能体的实际回答；支持异步批量执行、进度跟踪与失败重跑。</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>逐题调IRS推理收集实际回答；推理不经执行网关(CON-10)；异步批量执行；进度跟踪；失败题重跑</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>SRS R-SWM-004</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>对接 II-08/EI-06 本地推理</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>F-SWM-06-04</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>答案对比与打分</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>R-SWM-004</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>将跑题收集的实际回答与用例预期答案按评分标准对比打分，支持规则匹配、LLM裁判（LLM-as-judge）与人工评判三种模式，按用例逐题配置；LLM裁判置信度低时标记待人工评判。</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>规则匹配(精确/关键词)；LLM-as-judge(本地模型裁判)；人工评判；逐题配置评分模式；置信度低转人工</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>SRS R-SWM-004</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>F-SWM-06-05</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>评分汇总与报告</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>R-SWM-004</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>按评分维度（稳定性/合规性/人设一致性）汇总各维度得分、通过率、人设漂移维度，对比历史基线与上次同题集得分，输出评测报告；报告含质量等级、薄弱用例与改进建议。</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>维度得分汇总(稳定性/合规性/人设一致性)；通过率/人设漂移维度；历史基线对比；版本演进对比；评测报告输出</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>SRS R-SWM-004</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>供 F-SWM-06-06 决策消费</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>F-SWM-06-06</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>迭代/淘汰决策与反馈闭环</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>R-SWM-004</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>对低效定义提出淘汰、对高价值定义提出迭代优化；反馈至M-SWM-02(驱动模板迭代)与M-SWM-05(驱动定义重建)形成闭环。</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>淘汰/迭代决策；反馈构建侧形成闭环</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>综合 F-SWM-06-01 线上有效性统计与 F-SWM-06-05 离线数据集评测报告，对低效定义提出淘汰、对高价值定义提出迭代优化，形成评测决策；反馈至 M-SWM-02（驱动模板迭代）与 M-SWM-05（驱动定义重建）形成闭环。</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>综合线上+离线双轨结论；淘汰/迭代决策；反馈M-SWM-02模板迭代；反馈M-SWM-05定义重建；闭环</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-004</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr"/>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>原 F-SWM-06-03 顺延而来</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-09 16:46:10
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件概要设计-模块功能拆分.xlsx
+++ b/公司项目/认知作战/文档/软件概要设计-模块功能拆分.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12420" tabRatio="600" firstSheet="2" activeTab="5" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12420" tabRatio="600" firstSheet="2" activeTab="7" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块清单总览" sheetId="1" state="visible" r:id="rId1"/>
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -199,8 +199,17 @@
     <font>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="37">
+  <fills count="40">
     <fill>
       <patternFill/>
     </fill>
@@ -415,6 +424,21 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00305496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -701,7 +725,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -725,6 +749,15 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="37" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="38" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="39" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7474,7 +7507,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -7487,926 +7520,926 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>层级</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>编号</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>名称</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>对应需求</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>职责简述</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>关键能力点（功能）</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>来源依据</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="132" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>①子系统</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>M-SWM-00</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>蜂群智能体子系统</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>R-SWM-001~004</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>执行层的「智能体定义与记忆中心」：根据人设(画像/账号属性)编写驱动智能体作业的提示词与记忆，将智能体定义(人设标签/提示词/记忆/作业策略)以agent_id同步下发至MC持存；承担智能体构建、评测、提示词与人设管理、记忆管理；不直接操作设备。</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="10" t="inlineStr">
         <is>
           <t>SRS §引言/SWM</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="10" t="inlineStr">
         <is>
           <t>R-SWM-001(提示词与人设管理)含人设标签、提示词模板库、场景适配调用三个异构关注点(元数据/文本资产/运行时决策)，故拆3模块；智能体定义组装与同步下发归构建模块(M-SWM-05)，迭代优化决策归评测模块(M-SWM-06)。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="49.5" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>②模块</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>M-SWM-01</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>人设标签管理（智能体人格定义中心）</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>R-SWM-001(人设)</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>为每个 agent_id 绑定人设标签(身份特征/立场倾向/语言风格/兴趣领域等画像属性)；人设挂 agent_id，经 agent_id↔account_id 1:1 绑定间接对应账号；不复制账号主数据。</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>F-SWM-01-01 人设标签绑定；F-SWM-01-02 人设标签体系维护</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>SRS R-SWM-001(人设)</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>R-SWM-001 的人设标签(元数据体系)与提示词(文本资产)、运行时选择是不同职责域，故拆。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="33" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>FR-SWM-001 的人设标签(元数据体系)与提示词(文本资产)、运行时选择是不同职责域，故拆。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>F-SWM-01-01</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>人设标签绑定</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>R-SWM-001</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>为每个 agent_id 绑定人设标签，标签涵盖身份特征、立场倾向、语言风格、兴趣领域等画像属性。</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>人设绑agent_id；画像属性涵盖</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-001</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr"/>
+      <c r="H4" s="8" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>F-SWM-01-02</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>人设标签体系维护</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>R-SWM-001</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>维护人设标签体系定义；人设标签冲突时提示人工裁定。</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>标签体系维护；冲突人工裁定</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-001</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6" ht="49.5" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>②模块</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>M-SWM-02</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>提示词模板库与版本管理（提示词资产管理）</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>R-SWM-001(资产)</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>建立提示词模板库并按用途/平台/目标分类管理；对提示词进行版本管理，以 agent_id 为主键索引，支持版本对比/回滚/变更记录。</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>F-SWM-02-01 提示词模板库分类管理；F-SWM-02-02 提示词版本管理</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>SRS R-SWM-001(资产)</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>R-SWM-001 的提示词模板库(文本资产)是独立关注点；版本管理横切于人设与提示词。</t>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>FR-SWM-001 的提示词模板库(文本资产)是独立关注点；版本管理横切于人设与提示词。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>F-SWM-02-01</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>提示词模板库分类管理</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>R-SWM-001</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>建立提示词模板库并按用途、平台、目标进行分类管理。</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>模板库；按用途/平台/目标分类</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-001</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8" ht="33" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>F-SWM-02-02</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>提示词版本管理</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>R-SWM-001</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>对提示词进行版本管理，以 agent_id 为主键索引，支持版本对比、回滚与变更记录；版本回滚失败时告警。</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>agent_id主键版本管理；对比/回滚/变更记录</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-001</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9" ht="49.5" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>②模块</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>M-SWM-03</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>提示词场景适配与动态调用（提示词运行时引擎）</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>R-SWM-001(运行时)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>按作业场景(人设标签/目标受众/当前态势)适配提示词，作业时动态调用并填充生成最终作业指令。</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>F-SWM-03-01 场景适配；F-SWM-03-02 动态调用与指令生成</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>SRS R-SWM-001(运行时)</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>R-SWM-001 的场景适配与动态调用是运行时决策关注点，与模板库资产管理分离。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="33" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>FR-SWM-001 的场景适配与动态调用是运行时决策关注点，与模板库资产管理分离。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>F-SWM-03-01</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>场景适配</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>R-SWM-001</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>按作业场景(人设标签/目标受众/当前态势)选择合适模板；模板填充失败时降级为默认模板。</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>场景适配模板；填充失败降级默认</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-001</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr"/>
+      <c r="H10" s="8" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>F-SWM-03-02</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>动态调用与指令生成</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>R-SWM-001</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>智能体作业时动态调用并填充提示词，生成最终作业指令。</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>动态调用填充；生成作业指令</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-001</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>对接 II-09</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="49.5" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>②模块</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>M-SWM-04</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>蜂群记忆管理（智能体记忆中枢）</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>R-SWM-002</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>实现智能体作业记忆的存储、场景沉淀、历史复用与个性化状态延续，使智能体长期行为符合人设且不断演进。</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>F-SWM-04-01 作业记忆存储；F-SWM-04-02 场景记忆沉淀；F-SWM-04-03 历史记忆复用；F-SWM-04-04 个性化状态延续</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>SRS R-SWM-002</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>对应 R-SWM-002，记忆存储/沉淀/复用/延续是同一记忆对象的生命周期环节，内聚不拆。</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="33" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>F-SWM-04-01</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>作业记忆存储</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>R-SWM-002</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>对智能体作业过程中的关键信息(已完成任务/互动对象/立场表达等)进行记忆存储。</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>关键信息记忆存储</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-002</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr"/>
+      <c r="H13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>F-SWM-04-02</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>场景记忆沉淀</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>R-SWM-002</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>将重复场景下的经验沉淀为场景记忆，形成可复用行为模式。</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>场景经验沉淀为模式</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-002</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr"/>
+      <c r="H14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>F-SWM-04-03</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>历史记忆复用</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>R-SWM-002</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>在相似作业中复用历史记忆，提升作业连贯性与效率。</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>相似作业复用历史记忆</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-002</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr"/>
+      <c r="H15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>F-SWM-04-04</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>个性化状态延续</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>R-SWM-002</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>基于记忆维持智能体个性化状态延续，使其长期行为符合人设且不断演进。</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>个性化状态延续；符合人设演进</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-002</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17" ht="82.5" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>②模块</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>M-SWM-05</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>智能体构建与定义下发（智能体装配工厂）</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>R-SWM-003</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>根据人设标签编写提示词与记忆初值、配置作业策略，组装为完整智能体定义并以 agent_id 为标识，经 II-15 同步至 MC 持存、供 OCC 作战编排引用。</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>F-SWM-05-01 智能体定义构建；F-SWM-05-02 账号绑定引用；F-SWM-05-03 同步至MC持存；F-SWM-05-04 OCC智能体节点定义来源</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>SRS R-SWM-003</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>对应 R-SWM-003，构建是装配链(编写初值+配置策略+组装+下发)，内聚不拆；吸收 R-SWM-001 中『组装与同步下发』能力作为定义交付出口。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="33" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>对应 R-SWM-003，构建是装配链(编写初值+配置策略+组装+下发)，内聚不拆；吸收 FR-SWM-001 中『组装与同步下发』能力作为定义交付出口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>F-SWM-05-01</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>智能体定义构建</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>R-SWM-003</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>按人设标签编写提示词初值与记忆初值并配置作业策略(目标/场景/边界)，组装为完整智能体定义，以全局唯一 agent_id 为标识。</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>人设+提示词初值+记忆初值+作业策略；agent_id标识</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G18" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-003</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19" ht="33" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="H18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>F-SWM-05-02</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>账号绑定引用</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>R-SWM-003</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>智能体定义与账号严格1:1绑定(agent_id↔account_id)，绑定关系由MC维护，本子系统构建时引用account_id。</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>agent_id↔account_id 1:1；构建时引用account_id</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-003</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>绑定关系归 MC</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="33" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>F-SWM-05-03</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>同步至MC持存</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>R-SWM-003</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>构建完成的智能体定义经II-15同步至MC持存，取得持存版本号；定义更新时以同一agent_id重新同步。</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>经II-15同步；取得版本号；更新重同步</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-003</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>对接 II-15</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>F-SWM-05-04</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>OCC智能体节点定义来源</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>R-SWM-003</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>构建出的智能体定义是OCC作战编排中智能体节点的定义来源。</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>作为OCC编排智能体节点定义来源</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-003</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H21" s="8" t="inlineStr">
         <is>
           <t>对接 II-11</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="49.5" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>②模块</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>M-SWM-06</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>智能体评测与迭代决策（智能体质量裁判）</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>R-SWM-004</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>对构建出的智能体基于作业效果反馈(来自MC可观测性)与人设一致性进行质量评测，淘汰低效定义、迭代优化高价值定义，形成「构建→评测→迭代」闭环。</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>F-SWM-06-01 有效性评测(线上MC作业效果统计)；F-SWM-06-02 评测数据集管理；F-SWM-06-03 批量跑题执行；F-SWM-06-04 答案对比与打分；F-SWM-06-05 评分汇总与报告；F-SWM-06-06 迭代/淘汰决策与反馈闭环</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>对构建出的智能体采用「线上效果 + 离线数据集」双轨评测，淘汰低效定义、迭代优化高价值定义，形成「构建→评测→迭代」闭环。</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>F-SWM-06-01 有效性评测；F-SWM-06-02 评测数据集管理；F-SWM-06-03 批量跑题执行；F-SWM-06-04 答案对比与打分；F-SWM-06-05 评分汇总与报告；F-SWM-06-06 迭代/淘汰决策与反馈闭环</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>SRS R-SWM-004</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>对应 R-SWM-004。06-01 为线上效果统计(触达/互动/完成率)；06-02~05 为离线数据集评测流程(录入题集→跑题→打分→汇总)，按流程环节拆4个功能；一在线一离线互补评估；06-06 综合双轨结论做决策与反馈。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="33" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>③功能</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>③功能</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>F-SWM-06-01</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>有效性评测</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>R-SWM-004</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>基于MC可观测性上报的作业效果数据(触达/互动/任务完成率)评测智能体有效性。</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>基于MC作业效果评测有效性</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>SRS R-SWM-004</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="H23" s="8" t="inlineStr">
         <is>
           <t>数据来自 R-MC-006</t>
         </is>
@@ -8450,11 +8483,11 @@
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>数据集是离线评测的可复现基准，固定题集可对不同版本反复评测对比演进</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="33" customHeight="1">
+          <t>数据集是离线评测的可复现基准</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>③功能</t>
@@ -8492,7 +8525,7 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>对接 II-08/EI-06 本地推理</t>
+          <t>对接 II-08/EI-06</t>
         </is>
       </c>
     </row>
@@ -8612,11 +8645,7 @@
           <t>SRS R-SWM-004</t>
         </is>
       </c>
-      <c r="H28" s="8" t="inlineStr">
-        <is>
-          <t>原 F-SWM-06-03 顺延而来</t>
-        </is>
-      </c>
+      <c r="H28" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9392,7 +9421,7 @@
           <t>③功能</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>F-OCC-03-01</t>
         </is>
@@ -9430,7 +9459,7 @@
           <t>③功能</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>F-OCC-03-02</t>
         </is>
@@ -9868,7 +9897,7 @@
           <t>③功能</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>F-OCC-06-01</t>
         </is>
@@ -9906,7 +9935,7 @@
           <t>③功能</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>F-OCC-06-02</t>
         </is>
@@ -9944,7 +9973,7 @@
           <t>③功能</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>F-OCC-06-03</t>
         </is>
@@ -9982,7 +10011,7 @@
           <t>③功能</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>F-OCC-06-04</t>
         </is>

</xml_diff>

<commit_message>
vault backup: 2026-07-09 17:16:30
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件概要设计-模块功能拆分.xlsx
+++ b/公司项目/认知作战/文档/软件概要设计-模块功能拆分.xlsx
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>浏览器 Profile 创建与 CDP 接入</t>
+          <t>浏览器 Profile 创建与 API 接入</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -4124,12 +4124,12 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>基于开源 BotBrowser 定制内核创建浏览器 Profile，经 CDP 向服务端注册，记录 Profile 标识、Chromium 内核版本、分组与标签。</t>
+          <t>经商用指纹浏览器 API 创建浏览器 Profile（下发指纹模板、代理、分组、标签），商用产品返回 Profile 标识与调试端口；记录 Profile 标识、内核版本、调试端口、分组与标签。</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Profile 创建；CDP 注册；分组与标签管理</t>
+          <t>调用商用API创建Profile；指纹模板/代理下发；返回调试端口(CDP)；记录Profile台账</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -4137,7 +4137,11 @@
           <t>SRS R-MC-001；CON-12</t>
         </is>
       </c>
-      <c r="H5" s="8" t="n"/>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>对接 EI-07 指纹浏览器服务接口</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -4274,7 +4278,7 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>浏览器 Profile 指纹固化</t>
+          <t>浏览器 Profile 指纹固化（经商用API）</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -4284,12 +4288,12 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Profile 创建时生成并固化 20+ 维渲染层指纹(Canvas/WebGL/字体/时区/Audio/UA)，使 Profile 长期呈现一致的设备身份；一Profile对应一套固化指纹与一账号身份。</t>
+          <t>经商用指纹浏览器 API 配置 Profile 指纹模板（Canvas/WebGL/字体/时区/Audio/UA 等 20+ 维），由商用产品生成并固化指纹，使 Profile 长期呈现一致的设备身份；一Profile对应一套固化指纹与一账号身份。</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>20+维指纹固化；指纹长期一致；一Profile一身份</t>
+          <t>20+维指纹模板经API下发；商用产品生成固化；指纹长期一致；一Profile一身份</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -4297,7 +4301,11 @@
           <t>SRS R-MC-001；CON-12</t>
         </is>
       </c>
-      <c r="H9" s="8" t="n"/>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>指纹生成与固化由商用产品负责</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -4596,7 +4604,7 @@
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>对单台及多台终端提供低延迟实时画面预览与输入控制，支持多终端同屏监控；移动端用 WebRTC、桌面端浏览器 Profile 用 RDP。</t>
+          <t>对单台及多台终端提供低延迟实时画面预览与输入控制，支持多终端同屏监控；移动端用 WebRTC、桌面端指纹浏览器 Profile 用商用 API 画面预览。</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
@@ -4670,7 +4678,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>桌面端 RDP 远控</t>
+          <t>桌面端商用 API 画面远控</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -4680,12 +4688,12 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>桌面端浏览器 Profile 基于 RDP 传输画面，鼠标点击与键盘输入映射为桌面事件；远控通道与任务执行通道相互分离。</t>
+          <t>桌面端指纹浏览器 Profile 经商用产品 API 获取页面/窗口画面预览流；鼠标点击与键盘输入经 CDP 注入为页面事件；远控通道与任务执行通道相互分离。</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>RDP画面传输；鼠标键盘映射；远控与执行通道分离</t>
+          <t>商用API画面预览流；CDP注入页面事件；远控与执行通道分离</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -4693,7 +4701,11 @@
           <t>SRS R-MC-002</t>
         </is>
       </c>
-      <c r="H19" s="8" t="n"/>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>对接 EI-07；替代原 RDP 方案</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -4916,12 +4928,12 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>两种模式按终端类型适配底层控制通道：移动端用 ADB/无障碍，桌面端浏览器Profile用 CDP；通道对上层透明。</t>
+          <t>两种模式按终端类型适配底层控制通道：移动端用 ADB/无障碍，桌面端浏览器Profile启动后用 CDP（经商用产品返回的调试端口）；通道对上层透明。</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>移动端ADB/无障碍；桌面端CDP；对上层透明</t>
+          <t>移动端ADB/无障碍；桌面端CDP(商用产品调试端口)；对上层透明</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -4929,7 +4941,7 @@
           <t>SRS R-MC-003</t>
         </is>
       </c>
-      <c r="H25" s="8" t="n"/>
+      <c r="H25" s="8" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">

</xml_diff>